<commit_message>
Upgrade version 4 20250114
</commit_message>
<xml_diff>
--- a/src/main/resources/static/Futures of Flowiee.xlsx
+++ b/src/main/resources/static/Futures of Flowiee.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\App\FW_PMS\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54C34C3F-4E27-49AF-9B9E-9B566F8AA4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC1C545-2927-49E7-9A9C-36FC84CBE0A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="3" xr2:uid="{7E065712-1017-4994-91F5-97AFA9456CE1}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="1136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1226" uniqueCount="1137">
   <si>
     <t>Quản lý người dùng</t>
   </si>
@@ -7845,6 +7845,9 @@
   </si>
   <si>
     <t>Default 0</t>
+  </si>
+  <si>
+    <t>Nang cap them</t>
   </si>
 </sst>
 </file>
@@ -12976,21 +12979,33 @@
       <c r="B172" s="12" t="s">
         <v>886</v>
       </c>
+      <c r="C172" s="11" t="s">
+        <v>1124</v>
+      </c>
     </row>
     <row r="173" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B173" s="12" t="s">
         <v>887</v>
       </c>
+      <c r="C173" s="11" t="s">
+        <v>1124</v>
+      </c>
     </row>
     <row r="174" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B174" s="12" t="s">
         <v>888</v>
       </c>
+      <c r="C174" s="11" t="s">
+        <v>1124</v>
+      </c>
     </row>
     <row r="175" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B175" s="12" t="s">
         <v>889</v>
       </c>
+      <c r="C175" s="11" t="s">
+        <v>1121</v>
+      </c>
     </row>
     <row r="176" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B176" s="12" t="s">
@@ -13009,6 +13024,9 @@
       <c r="B178" s="12" t="s">
         <v>892</v>
       </c>
+      <c r="C178" s="11" t="s">
+        <v>1124</v>
+      </c>
     </row>
     <row r="179" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B179" s="12" t="s">
@@ -13019,11 +13037,17 @@
       <c r="B180" s="12" t="s">
         <v>894</v>
       </c>
+      <c r="C180" s="11" t="s">
+        <v>1129</v>
+      </c>
     </row>
     <row r="181" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B181" s="12" t="s">
         <v>895</v>
       </c>
+      <c r="C181" s="11" t="s">
+        <v>1136</v>
+      </c>
     </row>
     <row r="182" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B182" s="12" t="s">
@@ -13033,6 +13057,9 @@
     <row r="183" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B183" s="12" t="s">
         <v>897</v>
+      </c>
+      <c r="C183" s="11" t="s">
+        <v>1121</v>
       </c>
     </row>
     <row r="184" spans="2:3" x14ac:dyDescent="0.3">

</xml_diff>